<commit_message>
Auto update: 2026-09-15 coffee data
</commit_message>
<xml_diff>
--- a/coffee_stocks_history.xlsx
+++ b/coffee_stocks_history.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C61"/>
+  <dimension ref="A1:C62"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1205,6 +1205,19 @@
         <v>-525</v>
       </c>
     </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="B62" t="n">
+        <v>217932</v>
+      </c>
+      <c r="C62" t="n">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Auto update: 2026-09-16 coffee data
</commit_message>
<xml_diff>
--- a/coffee_stocks_history.xlsx
+++ b/coffee_stocks_history.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C62"/>
+  <dimension ref="A1:C63"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1218,6 +1218,19 @@
         <v>0</v>
       </c>
     </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="B63" t="n">
+        <v>217646</v>
+      </c>
+      <c r="C63" t="n">
+        <v>-286</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Auto update: 2026-09-17 coffee data
</commit_message>
<xml_diff>
--- a/coffee_stocks_history.xlsx
+++ b/coffee_stocks_history.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C63"/>
+  <dimension ref="A1:C64"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1231,6 +1231,19 @@
         <v>-286</v>
       </c>
     </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B64" t="n">
+        <v>233479</v>
+      </c>
+      <c r="C64" t="n">
+        <v>15833</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Auto update: 2026-09-18 coffee data
</commit_message>
<xml_diff>
--- a/coffee_stocks_history.xlsx
+++ b/coffee_stocks_history.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C64"/>
+  <dimension ref="A1:C65"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1244,6 +1244,19 @@
         <v>15833</v>
       </c>
     </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B65" t="n">
+        <v>247887</v>
+      </c>
+      <c r="C65" t="n">
+        <v>14408</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Auto update: 2026-09-19 coffee data
</commit_message>
<xml_diff>
--- a/coffee_stocks_history.xlsx
+++ b/coffee_stocks_history.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C65"/>
+  <dimension ref="A1:C66"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1257,6 +1257,19 @@
         <v>14408</v>
       </c>
     </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B66" t="n">
+        <v>258415</v>
+      </c>
+      <c r="C66" t="n">
+        <v>10528</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Auto update: 2026-09-22 coffee data
</commit_message>
<xml_diff>
--- a/coffee_stocks_history.xlsx
+++ b/coffee_stocks_history.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C66"/>
+  <dimension ref="A1:C67"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1270,6 +1270,19 @@
         <v>10528</v>
       </c>
     </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="B67" t="n">
+        <v>253355</v>
+      </c>
+      <c r="C67" t="n">
+        <v>-5060</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Auto update: 2026-09-23 coffee data
</commit_message>
<xml_diff>
--- a/coffee_stocks_history.xlsx
+++ b/coffee_stocks_history.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C67"/>
+  <dimension ref="A1:C68"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1283,6 +1283,19 @@
         <v>-5060</v>
       </c>
     </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="B68" t="n">
+        <v>256678</v>
+      </c>
+      <c r="C68" t="n">
+        <v>3323</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Auto update: 2026-09-24 coffee data
</commit_message>
<xml_diff>
--- a/coffee_stocks_history.xlsx
+++ b/coffee_stocks_history.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C68"/>
+  <dimension ref="A1:C69"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1296,6 +1296,19 @@
         <v>3323</v>
       </c>
     </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+      <c r="B69" t="n">
+        <v>254480</v>
+      </c>
+      <c r="C69" t="n">
+        <v>-2198</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Auto update: 2026-09-25 coffee data
</commit_message>
<xml_diff>
--- a/coffee_stocks_history.xlsx
+++ b/coffee_stocks_history.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C69"/>
+  <dimension ref="A1:C70"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1309,6 +1309,19 @@
         <v>-2198</v>
       </c>
     </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="B70" t="n">
+        <v>254304</v>
+      </c>
+      <c r="C70" t="n">
+        <v>-176</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Auto update: 2026-09-26 coffee data
</commit_message>
<xml_diff>
--- a/coffee_stocks_history.xlsx
+++ b/coffee_stocks_history.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C70"/>
+  <dimension ref="A1:C71"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1322,6 +1322,19 @@
         <v>-176</v>
       </c>
     </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="B71" t="n">
+        <v>254304</v>
+      </c>
+      <c r="C71" t="n">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Auto update: 2026-09-30 coffee data
</commit_message>
<xml_diff>
--- a/coffee_stocks_history.xlsx
+++ b/coffee_stocks_history.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C71"/>
+  <dimension ref="A1:C72"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1335,6 +1335,19 @@
         <v>0</v>
       </c>
     </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+      <c r="B72" t="n">
+        <v>255721</v>
+      </c>
+      <c r="C72" t="n">
+        <v>1417</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Auto update: 2026-10-01 coffee data
</commit_message>
<xml_diff>
--- a/coffee_stocks_history.xlsx
+++ b/coffee_stocks_history.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C72"/>
+  <dimension ref="A1:C73"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1348,6 +1348,19 @@
         <v>1417</v>
       </c>
     </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="B73" t="n">
+        <v>260654</v>
+      </c>
+      <c r="C73" t="n">
+        <v>4933</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Auto update: 2026-10-02 coffee data
</commit_message>
<xml_diff>
--- a/coffee_stocks_history.xlsx
+++ b/coffee_stocks_history.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C73"/>
+  <dimension ref="A1:C74"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1361,6 +1361,19 @@
         <v>4933</v>
       </c>
     </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
+      <c r="B74" t="n">
+        <v>260364</v>
+      </c>
+      <c r="C74" t="n">
+        <v>-290</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Auto update: 2026-10-03 coffee data
</commit_message>
<xml_diff>
--- a/coffee_stocks_history.xlsx
+++ b/coffee_stocks_history.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C74"/>
+  <dimension ref="A1:C75"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1374,6 +1374,19 @@
         <v>-290</v>
       </c>
     </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+      <c r="B75" t="n">
+        <v>260239</v>
+      </c>
+      <c r="C75" t="n">
+        <v>-125</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Auto update: 2026-10-06 coffee data
</commit_message>
<xml_diff>
--- a/coffee_stocks_history.xlsx
+++ b/coffee_stocks_history.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C75"/>
+  <dimension ref="A1:C76"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1387,6 +1387,19 @@
         <v>-125</v>
       </c>
     </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>2026-10-05</t>
+        </is>
+      </c>
+      <c r="B76" t="n">
+        <v>259989</v>
+      </c>
+      <c r="C76" t="n">
+        <v>-250</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Auto update: 2026-10-07 coffee data
</commit_message>
<xml_diff>
--- a/coffee_stocks_history.xlsx
+++ b/coffee_stocks_history.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C76"/>
+  <dimension ref="A1:C77"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1400,6 +1400,19 @@
         <v>-250</v>
       </c>
     </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="B77" t="n">
+        <v>254527</v>
+      </c>
+      <c r="C77" t="n">
+        <v>-5462</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Auto update: 2026-10-08 coffee data
</commit_message>
<xml_diff>
--- a/coffee_stocks_history.xlsx
+++ b/coffee_stocks_history.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C77"/>
+  <dimension ref="A1:C78"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1413,6 +1413,19 @@
         <v>-5462</v>
       </c>
     </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="B78" t="n">
+        <v>253251</v>
+      </c>
+      <c r="C78" t="n">
+        <v>-1276</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Auto update: 2026-10-09 coffee data
</commit_message>
<xml_diff>
--- a/coffee_stocks_history.xlsx
+++ b/coffee_stocks_history.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C78"/>
+  <dimension ref="A1:C79"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1426,6 +1426,19 @@
         <v>-1276</v>
       </c>
     </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+      <c r="B79" t="n">
+        <v>252256</v>
+      </c>
+      <c r="C79" t="n">
+        <v>-995</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Auto update: 2026-10-10 coffee data
</commit_message>
<xml_diff>
--- a/coffee_stocks_history.xlsx
+++ b/coffee_stocks_history.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C79"/>
+  <dimension ref="A1:C80"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1439,6 +1439,19 @@
         <v>-995</v>
       </c>
     </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="B80" t="n">
+        <v>252006</v>
+      </c>
+      <c r="C80" t="n">
+        <v>-250</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Auto update: 2026-10-13 coffee data
</commit_message>
<xml_diff>
--- a/coffee_stocks_history.xlsx
+++ b/coffee_stocks_history.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C80"/>
+  <dimension ref="A1:C81"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1452,6 +1452,19 @@
         <v>-250</v>
       </c>
     </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>2026-10-12</t>
+        </is>
+      </c>
+      <c r="B81" t="n">
+        <v>250171</v>
+      </c>
+      <c r="C81" t="n">
+        <v>-1835</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Auto update: 2026-10-14 coffee data
</commit_message>
<xml_diff>
--- a/coffee_stocks_history.xlsx
+++ b/coffee_stocks_history.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C81"/>
+  <dimension ref="A1:C82"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1465,6 +1465,19 @@
         <v>-1835</v>
       </c>
     </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+      <c r="B82" t="n">
+        <v>246856</v>
+      </c>
+      <c r="C82" t="n">
+        <v>-3315</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Auto update: 2026-10-15 coffee data
</commit_message>
<xml_diff>
--- a/coffee_stocks_history.xlsx
+++ b/coffee_stocks_history.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C82"/>
+  <dimension ref="A1:C83"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1478,6 +1478,19 @@
         <v>-3315</v>
       </c>
     </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B83" t="n">
+        <v>241947</v>
+      </c>
+      <c r="C83" t="n">
+        <v>-4909</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Auto update: 2026-10-16 coffee data
</commit_message>
<xml_diff>
--- a/coffee_stocks_history.xlsx
+++ b/coffee_stocks_history.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C83"/>
+  <dimension ref="A1:C84"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1491,6 +1491,19 @@
         <v>-4909</v>
       </c>
     </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="B84" t="n">
+        <v>238976</v>
+      </c>
+      <c r="C84" t="n">
+        <v>-2971</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Auto update: 2026-10-17 coffee data
</commit_message>
<xml_diff>
--- a/coffee_stocks_history.xlsx
+++ b/coffee_stocks_history.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C84"/>
+  <dimension ref="A1:C85"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1504,6 +1504,19 @@
         <v>-2971</v>
       </c>
     </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="B85" t="n">
+        <v>240767</v>
+      </c>
+      <c r="C85" t="n">
+        <v>1791</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Auto update: 2026-10-20 coffee data
</commit_message>
<xml_diff>
--- a/coffee_stocks_history.xlsx
+++ b/coffee_stocks_history.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C85"/>
+  <dimension ref="A1:C86"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1517,6 +1517,19 @@
         <v>1791</v>
       </c>
     </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>2026-10-19</t>
+        </is>
+      </c>
+      <c r="B86" t="n">
+        <v>239852</v>
+      </c>
+      <c r="C86" t="n">
+        <v>-915</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Auto update: 2026-10-21 coffee data
</commit_message>
<xml_diff>
--- a/coffee_stocks_history.xlsx
+++ b/coffee_stocks_history.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C86"/>
+  <dimension ref="A1:C87"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1530,6 +1530,19 @@
         <v>-915</v>
       </c>
     </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="B87" t="n">
+        <v>234901</v>
+      </c>
+      <c r="C87" t="n">
+        <v>-4951</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Auto update: 2026-10-22 coffee data
</commit_message>
<xml_diff>
--- a/coffee_stocks_history.xlsx
+++ b/coffee_stocks_history.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C87"/>
+  <dimension ref="A1:C88"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1543,6 +1543,19 @@
         <v>-4951</v>
       </c>
     </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="B88" t="n">
+        <v>239748</v>
+      </c>
+      <c r="C88" t="n">
+        <v>4847</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Auto update: 2026-10-23 coffee data
</commit_message>
<xml_diff>
--- a/coffee_stocks_history.xlsx
+++ b/coffee_stocks_history.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C88"/>
+  <dimension ref="A1:C89"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1556,6 +1556,19 @@
         <v>4847</v>
       </c>
     </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>2026-10-22</t>
+        </is>
+      </c>
+      <c r="B89" t="n">
+        <v>234433</v>
+      </c>
+      <c r="C89" t="n">
+        <v>-5315</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Auto update: 2026-10-24 coffee data
</commit_message>
<xml_diff>
--- a/coffee_stocks_history.xlsx
+++ b/coffee_stocks_history.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C89"/>
+  <dimension ref="A1:C90"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1569,6 +1569,19 @@
         <v>-5315</v>
       </c>
     </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="B90" t="n">
+        <v>227978</v>
+      </c>
+      <c r="C90" t="n">
+        <v>-6455</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Auto update: 2026-10-27 coffee data
</commit_message>
<xml_diff>
--- a/coffee_stocks_history.xlsx
+++ b/coffee_stocks_history.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C90"/>
+  <dimension ref="A1:C91"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1582,6 +1582,19 @@
         <v>-6455</v>
       </c>
     </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>2026-10-26</t>
+        </is>
+      </c>
+      <c r="B91" t="n">
+        <v>225610</v>
+      </c>
+      <c r="C91" t="n">
+        <v>-2368</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Auto update: 2026-10-28 coffee data
</commit_message>
<xml_diff>
--- a/coffee_stocks_history.xlsx
+++ b/coffee_stocks_history.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C91"/>
+  <dimension ref="A1:C92"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1595,6 +1595,19 @@
         <v>-2368</v>
       </c>
     </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>2026-10-27</t>
+        </is>
+      </c>
+      <c r="B92" t="n">
+        <v>224822</v>
+      </c>
+      <c r="C92" t="n">
+        <v>-788</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Auto update: 2026-10-30 coffee data
</commit_message>
<xml_diff>
--- a/coffee_stocks_history.xlsx
+++ b/coffee_stocks_history.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C92"/>
+  <dimension ref="A1:C93"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1608,6 +1608,19 @@
         <v>-788</v>
       </c>
     </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>2026-10-29</t>
+        </is>
+      </c>
+      <c r="B93" t="n">
+        <v>225068</v>
+      </c>
+      <c r="C93" t="n">
+        <v>246</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>